<commit_message>
Add conditional formatting (green/yellow/red) and 5 embedded charts to workbook
Agent-Logs-Url: https://github.com/pramod51/medplus/sessions/2ead48c8-aee5-4904-98e5-777f42b985e7

Co-authored-by: ydvashwani <47135442+ydvashwani@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Semiconductor_WC_Benchmarking.xlsx
+++ b/Semiconductor_WC_Benchmarking.xlsx
@@ -12,8 +12,9 @@
     <sheet name="Efficiency_Metrics" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Scoring_Ranking" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Benchmark_Analysis" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Cash_Release" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Dashboard" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Charts" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Cash_Release" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Dashboard" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26,7 +27,7 @@
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -62,6 +63,10 @@
       <i val="1"/>
       <color rgb="00595959"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="9">
@@ -107,7 +112,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -121,11 +126,39 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -217,6 +250,38 @@
     <xf numFmtId="3" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -291,6 +356,719 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Cash Conversion Cycle (CCC) — Peer Comparison</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="bar"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <v>CCC (days)</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Charts'!$A$4:$A$13</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Charts'!$E$4:$E$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <overlap val="-10"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <numFmt formatCode="0" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Days</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>DSO vs DIO vs DPO — Working Capital Days Breakdown</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="bar"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <v>DSO</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Charts'!$A$4:$A$13</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Charts'!$B$4:$B$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <v>DIO</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Charts'!$A$4:$A$13</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Charts'!$C$4:$C$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <v>DPO</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Charts'!$A$4:$A$13</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Charts'!$D$4:$D$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <overlap val="-10"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <numFmt formatCode="0" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Days</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>AR Turns vs Inventory Turns — Efficiency Comparison</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="bar"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <v>AR Turns</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Charts'!$A$4:$A$13</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Charts'!$F$4:$F$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <v>Inv Turns</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Charts'!$A$4:$A$13</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Charts'!$G$4:$G$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <overlap val="-10"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <numFmt formatCode="0" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Turns</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Cash Release Potential by Component ($M)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="stacked"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <v>AR Release</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Charts'!$A$4:$A$13</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Charts'!$L$4:$L$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <v>Inv Release</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Charts'!$A$4:$A$13</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Charts'!$M$4:$M$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <v>AP Release</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Charts'!$A$4:$A$13</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Charts'!$N$4:$N$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>$M</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Overall Rank — Composite Scorecard (1 = Best)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <v>Overall Rank</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Charts'!$A$4:$A$13</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Charts'!$K$4:$K$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <overlap val="-10"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <numFmt formatCode="0" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Rank (lower=better)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>15</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7920000" cy="5040000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>15</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7920000" cy="5040000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>46</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7920000" cy="5040000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="3" name="Chart 3"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>46</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7920000" cy="5040000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="4" name="Chart 4"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>77</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7920000" cy="5040000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="5" name="Chart 5"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId5"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1842,6 +2620,10 @@
           <t>Best-in-Class WC/Rev  →</t>
         </is>
       </c>
+      <c r="B14" s="31" t="n"/>
+      <c r="C14" s="31" t="n"/>
+      <c r="D14" s="31" t="n"/>
+      <c r="E14" s="32" t="n"/>
       <c r="F14" s="19">
         <f>MIN(F3:F12)</f>
         <v/>
@@ -1853,6 +2635,10 @@
           <t>Best-in-Class NWC/Rev →</t>
         </is>
       </c>
+      <c r="B15" s="31" t="n"/>
+      <c r="C15" s="31" t="n"/>
+      <c r="D15" s="31" t="n"/>
+      <c r="E15" s="32" t="n"/>
       <c r="K15" s="19">
         <f>MIN(K3:K12)</f>
         <v/>
@@ -1864,6 +2650,10 @@
           <t>Peer-Avg Current Ratio →</t>
         </is>
       </c>
+      <c r="B16" s="31" t="n"/>
+      <c r="C16" s="31" t="n"/>
+      <c r="D16" s="31" t="n"/>
+      <c r="E16" s="32" t="n"/>
       <c r="L16" s="20">
         <f>AVERAGE(L3:L12)</f>
         <v/>
@@ -1875,6 +2665,10 @@
           <t>Peer-Avg Quick Ratio   →</t>
         </is>
       </c>
+      <c r="B17" s="31" t="n"/>
+      <c r="C17" s="31" t="n"/>
+      <c r="D17" s="31" t="n"/>
+      <c r="E17" s="32" t="n"/>
       <c r="M17" s="20">
         <f>AVERAGE(M3:M12)</f>
         <v/>
@@ -1896,6 +2690,102 @@
     <mergeCell ref="A14:E14"/>
     <mergeCell ref="A17:E17"/>
   </mergeCells>
+  <conditionalFormatting sqref="D3:D12">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F3:F12">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J3:J12">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K3:K12">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L3:L12">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M3:M12">
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N3:N12">
+    <cfRule type="colorScale" priority="7">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O3:O12">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2798,6 +3688,12 @@
           <t>Best DSO (Min):</t>
         </is>
       </c>
+      <c r="B14" s="31" t="n"/>
+      <c r="C14" s="31" t="n"/>
+      <c r="D14" s="31" t="n"/>
+      <c r="E14" s="31" t="n"/>
+      <c r="F14" s="31" t="n"/>
+      <c r="G14" s="32" t="n"/>
       <c r="H14" s="23">
         <f>MIN(H3:H12)</f>
         <v/>
@@ -2809,6 +3705,12 @@
           <t>Best AR Turns (Max):</t>
         </is>
       </c>
+      <c r="B15" s="31" t="n"/>
+      <c r="C15" s="31" t="n"/>
+      <c r="D15" s="31" t="n"/>
+      <c r="E15" s="31" t="n"/>
+      <c r="F15" s="31" t="n"/>
+      <c r="G15" s="32" t="n"/>
       <c r="I15" s="23">
         <f>MAX(I3:I12)</f>
         <v/>
@@ -2820,6 +3722,12 @@
           <t>Best DIO (Min):</t>
         </is>
       </c>
+      <c r="B16" s="31" t="n"/>
+      <c r="C16" s="31" t="n"/>
+      <c r="D16" s="31" t="n"/>
+      <c r="E16" s="31" t="n"/>
+      <c r="F16" s="31" t="n"/>
+      <c r="G16" s="32" t="n"/>
       <c r="J16" s="23">
         <f>MIN(J3:J12)</f>
         <v/>
@@ -2831,6 +3739,12 @@
           <t>Best Inv Turns (Max):</t>
         </is>
       </c>
+      <c r="B17" s="31" t="n"/>
+      <c r="C17" s="31" t="n"/>
+      <c r="D17" s="31" t="n"/>
+      <c r="E17" s="31" t="n"/>
+      <c r="F17" s="31" t="n"/>
+      <c r="G17" s="32" t="n"/>
       <c r="K17" s="23">
         <f>MAX(K3:K12)</f>
         <v/>
@@ -2842,6 +3756,12 @@
           <t>Best DPO (Max):</t>
         </is>
       </c>
+      <c r="B18" s="31" t="n"/>
+      <c r="C18" s="31" t="n"/>
+      <c r="D18" s="31" t="n"/>
+      <c r="E18" s="31" t="n"/>
+      <c r="F18" s="31" t="n"/>
+      <c r="G18" s="32" t="n"/>
       <c r="L18" s="23">
         <f>MAX(L3:L12)</f>
         <v/>
@@ -2853,6 +3773,12 @@
           <t>Best CCC (Min):</t>
         </is>
       </c>
+      <c r="B19" s="31" t="n"/>
+      <c r="C19" s="31" t="n"/>
+      <c r="D19" s="31" t="n"/>
+      <c r="E19" s="31" t="n"/>
+      <c r="F19" s="31" t="n"/>
+      <c r="G19" s="32" t="n"/>
       <c r="M19" s="23">
         <f>MIN(M3:M12)</f>
         <v/>
@@ -2864,6 +3790,12 @@
           <t>Best CRR (Max):</t>
         </is>
       </c>
+      <c r="B20" s="31" t="n"/>
+      <c r="C20" s="31" t="n"/>
+      <c r="D20" s="31" t="n"/>
+      <c r="E20" s="31" t="n"/>
+      <c r="F20" s="31" t="n"/>
+      <c r="G20" s="32" t="n"/>
       <c r="N20" s="19">
         <f>MAX(N3:N12)</f>
         <v/>
@@ -2888,6 +3820,90 @@
     <mergeCell ref="A15:G15"/>
     <mergeCell ref="A19:G19"/>
   </mergeCells>
+  <conditionalFormatting sqref="H3:H12">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I3:I12">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J3:J12">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K3:K12">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L3:L12">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M3:M12">
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N3:N12">
+    <cfRule type="colorScale" priority="7">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3414,6 +4430,30 @@
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A14:J14"/>
   </mergeCells>
+  <conditionalFormatting sqref="H3:H12">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I3:I12">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4319,11 +5359,818 @@
     <mergeCell ref="A14:R14"/>
     <mergeCell ref="A1:R1"/>
   </mergeCells>
+  <conditionalFormatting sqref="F3:F12">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I3:I12">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L3:L12">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O3:O12">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R3:R12">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:S13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Semiconductor WC Benchmarking — Visual Analysis Charts (auto-refresh with source data)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="40" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>DSO
+(days)</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>DIO
+(days)</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>DPO
+(days)</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>CCC
+(days)</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>AR Turns</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Inv Turns</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>CRR (%)</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>WC/Rev (%)</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>NWC/Rev (%)</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Overall Rank</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>AR Release
+($M)</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Inv Release
+($M)</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>AP Release
+($M)</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>Total Release
+($M)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="33">
+        <f>Raw_Data!A3</f>
+        <v/>
+      </c>
+      <c r="B4" s="34">
+        <f>Efficiency_Metrics!H3</f>
+        <v/>
+      </c>
+      <c r="C4" s="34">
+        <f>Efficiency_Metrics!J3</f>
+        <v/>
+      </c>
+      <c r="D4" s="34">
+        <f>Efficiency_Metrics!L3</f>
+        <v/>
+      </c>
+      <c r="E4" s="34">
+        <f>Efficiency_Metrics!M3</f>
+        <v/>
+      </c>
+      <c r="F4" s="34">
+        <f>Efficiency_Metrics!I3</f>
+        <v/>
+      </c>
+      <c r="G4" s="34">
+        <f>Efficiency_Metrics!K3</f>
+        <v/>
+      </c>
+      <c r="H4" s="35">
+        <f>Efficiency_Metrics!N3</f>
+        <v/>
+      </c>
+      <c r="I4" s="35">
+        <f>WC_NWC!F3</f>
+        <v/>
+      </c>
+      <c r="J4" s="35">
+        <f>WC_NWC!K3</f>
+        <v/>
+      </c>
+      <c r="K4" s="36">
+        <f>Scoring_Ranking!I3</f>
+        <v/>
+      </c>
+      <c r="L4" s="37">
+        <f>Cash_Release!I3</f>
+        <v/>
+      </c>
+      <c r="M4" s="37">
+        <f>Cash_Release!N3</f>
+        <v/>
+      </c>
+      <c r="N4" s="37">
+        <f>Cash_Release!S3</f>
+        <v/>
+      </c>
+      <c r="O4" s="37">
+        <f>Cash_Release!T3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="38">
+        <f>Raw_Data!A4</f>
+        <v/>
+      </c>
+      <c r="B5" s="39">
+        <f>Efficiency_Metrics!H4</f>
+        <v/>
+      </c>
+      <c r="C5" s="39">
+        <f>Efficiency_Metrics!J4</f>
+        <v/>
+      </c>
+      <c r="D5" s="39">
+        <f>Efficiency_Metrics!L4</f>
+        <v/>
+      </c>
+      <c r="E5" s="39">
+        <f>Efficiency_Metrics!M4</f>
+        <v/>
+      </c>
+      <c r="F5" s="39">
+        <f>Efficiency_Metrics!I4</f>
+        <v/>
+      </c>
+      <c r="G5" s="39">
+        <f>Efficiency_Metrics!K4</f>
+        <v/>
+      </c>
+      <c r="H5" s="40">
+        <f>Efficiency_Metrics!N4</f>
+        <v/>
+      </c>
+      <c r="I5" s="40">
+        <f>WC_NWC!F4</f>
+        <v/>
+      </c>
+      <c r="J5" s="40">
+        <f>WC_NWC!K4</f>
+        <v/>
+      </c>
+      <c r="K5" s="41">
+        <f>Scoring_Ranking!I4</f>
+        <v/>
+      </c>
+      <c r="L5" s="42">
+        <f>Cash_Release!I4</f>
+        <v/>
+      </c>
+      <c r="M5" s="42">
+        <f>Cash_Release!N4</f>
+        <v/>
+      </c>
+      <c r="N5" s="42">
+        <f>Cash_Release!S4</f>
+        <v/>
+      </c>
+      <c r="O5" s="42">
+        <f>Cash_Release!T4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="33">
+        <f>Raw_Data!A5</f>
+        <v/>
+      </c>
+      <c r="B6" s="34">
+        <f>Efficiency_Metrics!H5</f>
+        <v/>
+      </c>
+      <c r="C6" s="34">
+        <f>Efficiency_Metrics!J5</f>
+        <v/>
+      </c>
+      <c r="D6" s="34">
+        <f>Efficiency_Metrics!L5</f>
+        <v/>
+      </c>
+      <c r="E6" s="34">
+        <f>Efficiency_Metrics!M5</f>
+        <v/>
+      </c>
+      <c r="F6" s="34">
+        <f>Efficiency_Metrics!I5</f>
+        <v/>
+      </c>
+      <c r="G6" s="34">
+        <f>Efficiency_Metrics!K5</f>
+        <v/>
+      </c>
+      <c r="H6" s="35">
+        <f>Efficiency_Metrics!N5</f>
+        <v/>
+      </c>
+      <c r="I6" s="35">
+        <f>WC_NWC!F5</f>
+        <v/>
+      </c>
+      <c r="J6" s="35">
+        <f>WC_NWC!K5</f>
+        <v/>
+      </c>
+      <c r="K6" s="36">
+        <f>Scoring_Ranking!I5</f>
+        <v/>
+      </c>
+      <c r="L6" s="37">
+        <f>Cash_Release!I5</f>
+        <v/>
+      </c>
+      <c r="M6" s="37">
+        <f>Cash_Release!N5</f>
+        <v/>
+      </c>
+      <c r="N6" s="37">
+        <f>Cash_Release!S5</f>
+        <v/>
+      </c>
+      <c r="O6" s="37">
+        <f>Cash_Release!T5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="38">
+        <f>Raw_Data!A6</f>
+        <v/>
+      </c>
+      <c r="B7" s="39">
+        <f>Efficiency_Metrics!H6</f>
+        <v/>
+      </c>
+      <c r="C7" s="39">
+        <f>Efficiency_Metrics!J6</f>
+        <v/>
+      </c>
+      <c r="D7" s="39">
+        <f>Efficiency_Metrics!L6</f>
+        <v/>
+      </c>
+      <c r="E7" s="39">
+        <f>Efficiency_Metrics!M6</f>
+        <v/>
+      </c>
+      <c r="F7" s="39">
+        <f>Efficiency_Metrics!I6</f>
+        <v/>
+      </c>
+      <c r="G7" s="39">
+        <f>Efficiency_Metrics!K6</f>
+        <v/>
+      </c>
+      <c r="H7" s="40">
+        <f>Efficiency_Metrics!N6</f>
+        <v/>
+      </c>
+      <c r="I7" s="40">
+        <f>WC_NWC!F6</f>
+        <v/>
+      </c>
+      <c r="J7" s="40">
+        <f>WC_NWC!K6</f>
+        <v/>
+      </c>
+      <c r="K7" s="41">
+        <f>Scoring_Ranking!I6</f>
+        <v/>
+      </c>
+      <c r="L7" s="42">
+        <f>Cash_Release!I6</f>
+        <v/>
+      </c>
+      <c r="M7" s="42">
+        <f>Cash_Release!N6</f>
+        <v/>
+      </c>
+      <c r="N7" s="42">
+        <f>Cash_Release!S6</f>
+        <v/>
+      </c>
+      <c r="O7" s="42">
+        <f>Cash_Release!T6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="33">
+        <f>Raw_Data!A7</f>
+        <v/>
+      </c>
+      <c r="B8" s="34">
+        <f>Efficiency_Metrics!H7</f>
+        <v/>
+      </c>
+      <c r="C8" s="34">
+        <f>Efficiency_Metrics!J7</f>
+        <v/>
+      </c>
+      <c r="D8" s="34">
+        <f>Efficiency_Metrics!L7</f>
+        <v/>
+      </c>
+      <c r="E8" s="34">
+        <f>Efficiency_Metrics!M7</f>
+        <v/>
+      </c>
+      <c r="F8" s="34">
+        <f>Efficiency_Metrics!I7</f>
+        <v/>
+      </c>
+      <c r="G8" s="34">
+        <f>Efficiency_Metrics!K7</f>
+        <v/>
+      </c>
+      <c r="H8" s="35">
+        <f>Efficiency_Metrics!N7</f>
+        <v/>
+      </c>
+      <c r="I8" s="35">
+        <f>WC_NWC!F7</f>
+        <v/>
+      </c>
+      <c r="J8" s="35">
+        <f>WC_NWC!K7</f>
+        <v/>
+      </c>
+      <c r="K8" s="36">
+        <f>Scoring_Ranking!I7</f>
+        <v/>
+      </c>
+      <c r="L8" s="37">
+        <f>Cash_Release!I7</f>
+        <v/>
+      </c>
+      <c r="M8" s="37">
+        <f>Cash_Release!N7</f>
+        <v/>
+      </c>
+      <c r="N8" s="37">
+        <f>Cash_Release!S7</f>
+        <v/>
+      </c>
+      <c r="O8" s="37">
+        <f>Cash_Release!T7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="38">
+        <f>Raw_Data!A8</f>
+        <v/>
+      </c>
+      <c r="B9" s="39">
+        <f>Efficiency_Metrics!H8</f>
+        <v/>
+      </c>
+      <c r="C9" s="39">
+        <f>Efficiency_Metrics!J8</f>
+        <v/>
+      </c>
+      <c r="D9" s="39">
+        <f>Efficiency_Metrics!L8</f>
+        <v/>
+      </c>
+      <c r="E9" s="39">
+        <f>Efficiency_Metrics!M8</f>
+        <v/>
+      </c>
+      <c r="F9" s="39">
+        <f>Efficiency_Metrics!I8</f>
+        <v/>
+      </c>
+      <c r="G9" s="39">
+        <f>Efficiency_Metrics!K8</f>
+        <v/>
+      </c>
+      <c r="H9" s="40">
+        <f>Efficiency_Metrics!N8</f>
+        <v/>
+      </c>
+      <c r="I9" s="40">
+        <f>WC_NWC!F8</f>
+        <v/>
+      </c>
+      <c r="J9" s="40">
+        <f>WC_NWC!K8</f>
+        <v/>
+      </c>
+      <c r="K9" s="41">
+        <f>Scoring_Ranking!I8</f>
+        <v/>
+      </c>
+      <c r="L9" s="42">
+        <f>Cash_Release!I8</f>
+        <v/>
+      </c>
+      <c r="M9" s="42">
+        <f>Cash_Release!N8</f>
+        <v/>
+      </c>
+      <c r="N9" s="42">
+        <f>Cash_Release!S8</f>
+        <v/>
+      </c>
+      <c r="O9" s="42">
+        <f>Cash_Release!T8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="33">
+        <f>Raw_Data!A9</f>
+        <v/>
+      </c>
+      <c r="B10" s="34">
+        <f>Efficiency_Metrics!H9</f>
+        <v/>
+      </c>
+      <c r="C10" s="34">
+        <f>Efficiency_Metrics!J9</f>
+        <v/>
+      </c>
+      <c r="D10" s="34">
+        <f>Efficiency_Metrics!L9</f>
+        <v/>
+      </c>
+      <c r="E10" s="34">
+        <f>Efficiency_Metrics!M9</f>
+        <v/>
+      </c>
+      <c r="F10" s="34">
+        <f>Efficiency_Metrics!I9</f>
+        <v/>
+      </c>
+      <c r="G10" s="34">
+        <f>Efficiency_Metrics!K9</f>
+        <v/>
+      </c>
+      <c r="H10" s="35">
+        <f>Efficiency_Metrics!N9</f>
+        <v/>
+      </c>
+      <c r="I10" s="35">
+        <f>WC_NWC!F9</f>
+        <v/>
+      </c>
+      <c r="J10" s="35">
+        <f>WC_NWC!K9</f>
+        <v/>
+      </c>
+      <c r="K10" s="36">
+        <f>Scoring_Ranking!I9</f>
+        <v/>
+      </c>
+      <c r="L10" s="37">
+        <f>Cash_Release!I9</f>
+        <v/>
+      </c>
+      <c r="M10" s="37">
+        <f>Cash_Release!N9</f>
+        <v/>
+      </c>
+      <c r="N10" s="37">
+        <f>Cash_Release!S9</f>
+        <v/>
+      </c>
+      <c r="O10" s="37">
+        <f>Cash_Release!T9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="38">
+        <f>Raw_Data!A10</f>
+        <v/>
+      </c>
+      <c r="B11" s="39">
+        <f>Efficiency_Metrics!H10</f>
+        <v/>
+      </c>
+      <c r="C11" s="39">
+        <f>Efficiency_Metrics!J10</f>
+        <v/>
+      </c>
+      <c r="D11" s="39">
+        <f>Efficiency_Metrics!L10</f>
+        <v/>
+      </c>
+      <c r="E11" s="39">
+        <f>Efficiency_Metrics!M10</f>
+        <v/>
+      </c>
+      <c r="F11" s="39">
+        <f>Efficiency_Metrics!I10</f>
+        <v/>
+      </c>
+      <c r="G11" s="39">
+        <f>Efficiency_Metrics!K10</f>
+        <v/>
+      </c>
+      <c r="H11" s="40">
+        <f>Efficiency_Metrics!N10</f>
+        <v/>
+      </c>
+      <c r="I11" s="40">
+        <f>WC_NWC!F10</f>
+        <v/>
+      </c>
+      <c r="J11" s="40">
+        <f>WC_NWC!K10</f>
+        <v/>
+      </c>
+      <c r="K11" s="41">
+        <f>Scoring_Ranking!I10</f>
+        <v/>
+      </c>
+      <c r="L11" s="42">
+        <f>Cash_Release!I10</f>
+        <v/>
+      </c>
+      <c r="M11" s="42">
+        <f>Cash_Release!N10</f>
+        <v/>
+      </c>
+      <c r="N11" s="42">
+        <f>Cash_Release!S10</f>
+        <v/>
+      </c>
+      <c r="O11" s="42">
+        <f>Cash_Release!T10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="33">
+        <f>Raw_Data!A11</f>
+        <v/>
+      </c>
+      <c r="B12" s="34">
+        <f>Efficiency_Metrics!H11</f>
+        <v/>
+      </c>
+      <c r="C12" s="34">
+        <f>Efficiency_Metrics!J11</f>
+        <v/>
+      </c>
+      <c r="D12" s="34">
+        <f>Efficiency_Metrics!L11</f>
+        <v/>
+      </c>
+      <c r="E12" s="34">
+        <f>Efficiency_Metrics!M11</f>
+        <v/>
+      </c>
+      <c r="F12" s="34">
+        <f>Efficiency_Metrics!I11</f>
+        <v/>
+      </c>
+      <c r="G12" s="34">
+        <f>Efficiency_Metrics!K11</f>
+        <v/>
+      </c>
+      <c r="H12" s="35">
+        <f>Efficiency_Metrics!N11</f>
+        <v/>
+      </c>
+      <c r="I12" s="35">
+        <f>WC_NWC!F11</f>
+        <v/>
+      </c>
+      <c r="J12" s="35">
+        <f>WC_NWC!K11</f>
+        <v/>
+      </c>
+      <c r="K12" s="36">
+        <f>Scoring_Ranking!I11</f>
+        <v/>
+      </c>
+      <c r="L12" s="37">
+        <f>Cash_Release!I11</f>
+        <v/>
+      </c>
+      <c r="M12" s="37">
+        <f>Cash_Release!N11</f>
+        <v/>
+      </c>
+      <c r="N12" s="37">
+        <f>Cash_Release!S11</f>
+        <v/>
+      </c>
+      <c r="O12" s="37">
+        <f>Cash_Release!T11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="38">
+        <f>Raw_Data!A12</f>
+        <v/>
+      </c>
+      <c r="B13" s="39">
+        <f>Efficiency_Metrics!H12</f>
+        <v/>
+      </c>
+      <c r="C13" s="39">
+        <f>Efficiency_Metrics!J12</f>
+        <v/>
+      </c>
+      <c r="D13" s="39">
+        <f>Efficiency_Metrics!L12</f>
+        <v/>
+      </c>
+      <c r="E13" s="39">
+        <f>Efficiency_Metrics!M12</f>
+        <v/>
+      </c>
+      <c r="F13" s="39">
+        <f>Efficiency_Metrics!I12</f>
+        <v/>
+      </c>
+      <c r="G13" s="39">
+        <f>Efficiency_Metrics!K12</f>
+        <v/>
+      </c>
+      <c r="H13" s="40">
+        <f>Efficiency_Metrics!N12</f>
+        <v/>
+      </c>
+      <c r="I13" s="40">
+        <f>WC_NWC!F12</f>
+        <v/>
+      </c>
+      <c r="J13" s="40">
+        <f>WC_NWC!K12</f>
+        <v/>
+      </c>
+      <c r="K13" s="41">
+        <f>Scoring_Ranking!I12</f>
+        <v/>
+      </c>
+      <c r="L13" s="42">
+        <f>Cash_Release!I12</f>
+        <v/>
+      </c>
+      <c r="M13" s="42">
+        <f>Cash_Release!N12</f>
+        <v/>
+      </c>
+      <c r="N13" s="42">
+        <f>Cash_Release!S12</f>
+        <v/>
+      </c>
+      <c r="O13" s="42">
+        <f>Cash_Release!T12</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:S1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5313,6 +7160,13 @@
           <t>TOTAL All 10 Companies (MAX(…,0) ensures below-target contributes $0):</t>
         </is>
       </c>
+      <c r="B14" s="31" t="n"/>
+      <c r="C14" s="31" t="n"/>
+      <c r="D14" s="31" t="n"/>
+      <c r="E14" s="31" t="n"/>
+      <c r="F14" s="31" t="n"/>
+      <c r="G14" s="31" t="n"/>
+      <c r="H14" s="32" t="n"/>
       <c r="I14" s="24">
         <f>SUM(I3:I12)</f>
         <v/>
@@ -5335,6 +7189,13 @@
         <f>CONCATENATE("TOTAL Q3+Q4 Companies (",COUNTIF(B3:B12,"Q3")+COUNTIF(B3:B12,"Q4")," cos):  AR  |  Inv  |  AP  |  Combined")</f>
         <v/>
       </c>
+      <c r="B15" s="31" t="n"/>
+      <c r="C15" s="31" t="n"/>
+      <c r="D15" s="31" t="n"/>
+      <c r="E15" s="31" t="n"/>
+      <c r="F15" s="31" t="n"/>
+      <c r="G15" s="31" t="n"/>
+      <c r="H15" s="32" t="n"/>
       <c r="I15" s="26">
         <f>SUMIF(B3:B12,"Q3",I3:I12)+SUMIF(B3:B12,"Q4",I3:I12)</f>
         <v/>
@@ -5366,11 +7227,59 @@
     <mergeCell ref="A14:H14"/>
     <mergeCell ref="A15:H15"/>
   </mergeCells>
+  <conditionalFormatting sqref="I3:I12">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N3:N12">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S3:S12">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T3:T12">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5411,6 +7320,21 @@
           <t>SECTION A — Consolidated Metrics Per Company (all values pulled from analysis sheets)</t>
         </is>
       </c>
+      <c r="B3" s="31" t="n"/>
+      <c r="C3" s="31" t="n"/>
+      <c r="D3" s="31" t="n"/>
+      <c r="E3" s="31" t="n"/>
+      <c r="F3" s="31" t="n"/>
+      <c r="G3" s="31" t="n"/>
+      <c r="H3" s="31" t="n"/>
+      <c r="I3" s="31" t="n"/>
+      <c r="J3" s="31" t="n"/>
+      <c r="K3" s="31" t="n"/>
+      <c r="L3" s="31" t="n"/>
+      <c r="M3" s="31" t="n"/>
+      <c r="N3" s="31" t="n"/>
+      <c r="O3" s="31" t="n"/>
+      <c r="P3" s="32" t="n"/>
     </row>
     <row r="4" ht="45" customHeight="1">
       <c r="A4" s="28" t="inlineStr">
@@ -6171,6 +8095,21 @@
           <t>SECTION B — Peer Benchmark Summary (Best / Median / Worst — all formulas)</t>
         </is>
       </c>
+      <c r="B16" s="31" t="n"/>
+      <c r="C16" s="31" t="n"/>
+      <c r="D16" s="31" t="n"/>
+      <c r="E16" s="31" t="n"/>
+      <c r="F16" s="31" t="n"/>
+      <c r="G16" s="31" t="n"/>
+      <c r="H16" s="31" t="n"/>
+      <c r="I16" s="31" t="n"/>
+      <c r="J16" s="31" t="n"/>
+      <c r="K16" s="31" t="n"/>
+      <c r="L16" s="31" t="n"/>
+      <c r="M16" s="31" t="n"/>
+      <c r="N16" s="31" t="n"/>
+      <c r="O16" s="31" t="n"/>
+      <c r="P16" s="32" t="n"/>
     </row>
     <row r="17" ht="40" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
@@ -6523,6 +8462,21 @@
           <t>SECTION C — Cash Release Potential Summary (all values from Cash_Release sheet)</t>
         </is>
       </c>
+      <c r="B31" s="31" t="n"/>
+      <c r="C31" s="31" t="n"/>
+      <c r="D31" s="31" t="n"/>
+      <c r="E31" s="31" t="n"/>
+      <c r="F31" s="31" t="n"/>
+      <c r="G31" s="31" t="n"/>
+      <c r="H31" s="31" t="n"/>
+      <c r="I31" s="31" t="n"/>
+      <c r="J31" s="31" t="n"/>
+      <c r="K31" s="31" t="n"/>
+      <c r="L31" s="31" t="n"/>
+      <c r="M31" s="31" t="n"/>
+      <c r="N31" s="31" t="n"/>
+      <c r="O31" s="31" t="n"/>
+      <c r="P31" s="32" t="n"/>
     </row>
     <row r="32" ht="40" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
@@ -6616,6 +8570,162 @@
     <mergeCell ref="A3:P3"/>
     <mergeCell ref="A16:P16"/>
   </mergeCells>
+  <conditionalFormatting sqref="D5:D14">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E5:E14">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F5:F14">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G5:G14">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H5:H14">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I5:I14">
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J5:J14">
+    <cfRule type="colorScale" priority="7">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K5:K14">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L5:L14">
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M5:M14">
+    <cfRule type="colorScale" priority="10">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N5:N14">
+    <cfRule type="colorScale" priority="11">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O5:O14">
+    <cfRule type="colorScale" priority="12">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P5:P14">
+    <cfRule type="colorScale" priority="13">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>